<commit_message>
Add in a new metric to the Local Skills page to look in detail at apprenticeships and various cuts of app achievements.
</commit_message>
<xml_diff>
--- a/Data/3-1_DataTable/DataTable.xlsx
+++ b/Data/3-1_DataTable/DataTable.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://educationgovuk-my.sharepoint.com/personal/paul_james_education_gov_uk/Documents/Documents/RProjects/lsip_dashboard/Data/3-1_DataTable/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="20" documentId="13_ncr:1_{BB966AC7-D478-46F4-96D8-4ADE6513DE0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7DEE3EBA-6B8C-41C5-92E4-ED52225FAEF6}"/>
+  <xr:revisionPtr revIDLastSave="33" documentId="13_ncr:1_{BB966AC7-D478-46F4-96D8-4ADE6513DE0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{69B9780C-8328-4DBA-AA11-102CC5B63905}"/>
   <bookViews>
-    <workbookView xWindow="1820" yWindow="20" windowWidth="20660" windowHeight="14300" xr2:uid="{677CE7B9-0003-4845-87B7-4FABD7ACD82F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{677CE7B9-0003-4845-87B7-4FABD7ACD82F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="44">
   <si>
     <t>Data​</t>
   </si>
@@ -162,13 +162,19 @@
   </si>
   <si>
     <t>July 2025 - June 2026 (TBC)</t>
+  </si>
+  <si>
+    <t>&lt;a href='https://explore-education-statistics.service.gov.uk/find-statistics/apprenticeships/2024-25'&gt;Individualised Learner Record&lt;/a&gt;</t>
+  </si>
+  <si>
+    <t>Apprenticeship achievements by level, SSA, age and standard</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -196,6 +202,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -214,18 +228,21 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -538,7 +555,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6050695-7AD5-4EAF-ACCC-796FB129457A}">
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="86.7265625" customWidth="1"/>
@@ -546,7 +563,7 @@
     <col min="3" max="3" width="27.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="41" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="41" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -560,7 +577,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="27" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>19</v>
       </c>
@@ -574,7 +591,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="125" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" ht="125" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>18</v>
       </c>
@@ -588,7 +605,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
@@ -602,7 +619,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" ht="55" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>17</v>
       </c>
@@ -616,7 +633,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="83.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" ht="83.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
@@ -630,37 +647,38 @@
         <v>34</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
+    <row r="7" spans="1:8" ht="83.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C7" t="s">
+        <v>33</v>
+      </c>
+      <c r="D7" t="s">
+        <v>34</v>
+      </c>
+      <c r="H7" s="4"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
         <v>11</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B8" t="s">
         <v>4</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C8" t="s">
         <v>24</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D8" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
         <v>12</v>
-      </c>
-      <c r="B8" t="s">
-        <v>10</v>
-      </c>
-      <c r="C8" t="s">
-        <v>25</v>
-      </c>
-      <c r="D8" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>20</v>
       </c>
       <c r="B9" t="s">
         <v>10</v>
@@ -672,40 +690,40 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" t="s">
+        <v>10</v>
+      </c>
+      <c r="C10" t="s">
+        <v>25</v>
+      </c>
+      <c r="D10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
         <v>8</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B11" t="s">
         <v>9</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C11" t="s">
         <v>29</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D11" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
         <v>13</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B12" t="s">
         <v>28</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>14</v>
-      </c>
-      <c r="B12" t="s">
-        <v>27</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>35</v>
@@ -714,31 +732,45 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="2" t="s">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B14" t="s">
         <v>22</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C14" t="s">
         <v>38</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D14" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
         <v>15</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B15" t="s">
         <v>16</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C15" t="s">
         <v>23</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D15" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update destinations data to 24/25 data.
</commit_message>
<xml_diff>
--- a/Data/3-1_DataTable/DataTable.xlsx
+++ b/Data/3-1_DataTable/DataTable.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://educationgovuk-my.sharepoint.com/personal/paul_james_education_gov_uk/Documents/Documents/RProjects/lsip_dashboard/Data/3-1_DataTable/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="33" documentId="13_ncr:1_{BB966AC7-D478-46F4-96D8-4ADE6513DE0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{69B9780C-8328-4DBA-AA11-102CC5B63905}"/>
+  <xr:revisionPtr revIDLastSave="37" documentId="13_ncr:1_{BB966AC7-D478-46F4-96D8-4ADE6513DE0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{384C2CEE-B9BA-48A6-B893-1425A8C1C68F}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{677CE7B9-0003-4845-87B7-4FABD7ACD82F}"/>
   </bookViews>
@@ -143,12 +143,6 @@
     <t>Aug 2025 – Jul 2026 (Nov 26)</t>
   </si>
   <si>
-    <t>Aug 2023 -  Jul 2024 (22/23 learners) (26/03/26)</t>
-  </si>
-  <si>
-    <t>Aug 2023 -  Jul 2024 (22/23 learners) (tbc)</t>
-  </si>
-  <si>
     <t>April 2025 - Mar 2026 (TBC)</t>
   </si>
   <si>
@@ -168,6 +162,12 @@
   </si>
   <si>
     <t>Apprenticeship achievements by level, SSA, age and standard</t>
+  </si>
+  <si>
+    <t>Aug 2024 -  Jul 2025 (23/24 learners) (15/10/26)</t>
+  </si>
+  <si>
+    <t>Aug 2025 -  Jul 2026 (24/25 learners) (Oct 27)</t>
   </si>
 </sst>
 </file>
@@ -585,10 +585,10 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="125" customHeight="1" x14ac:dyDescent="0.35">
@@ -599,10 +599,10 @@
         <v>4</v>
       </c>
       <c r="C3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
@@ -613,10 +613,10 @@
         <v>4</v>
       </c>
       <c r="C4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D4" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="55" customHeight="1" x14ac:dyDescent="0.35">
@@ -649,10 +649,10 @@
     </row>
     <row r="7" spans="1:8" ht="83.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C7" t="s">
         <v>33</v>
@@ -673,7 +673,7 @@
         <v>24</v>
       </c>
       <c r="D8" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
@@ -726,10 +726,10 @@
         <v>28</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
@@ -740,10 +740,10 @@
         <v>27</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.35">
@@ -754,10 +754,10 @@
         <v>22</v>
       </c>
       <c r="C14" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D14" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Update documentation of business counts data (data itself was already updated in previous update thanks to the API)
</commit_message>
<xml_diff>
--- a/Data/3-1_DataTable/DataTable.xlsx
+++ b/Data/3-1_DataTable/DataTable.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://educationgovuk-my.sharepoint.com/personal/paul_james_education_gov_uk/Documents/Documents/RProjects/lsip_dashboard/Data/3-1_DataTable/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jscott8\R Projects\lsip_dashboard\Data\3-1_DataTable\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="37" documentId="13_ncr:1_{BB966AC7-D478-46F4-96D8-4ADE6513DE0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{384C2CEE-B9BA-48A6-B893-1425A8C1C68F}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{908255BD-55F3-4F2B-B2DD-9D3823E090BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{677CE7B9-0003-4845-87B7-4FABD7ACD82F}"/>
+    <workbookView xWindow="1530" yWindow="10690" windowWidth="22780" windowHeight="14540" xr2:uid="{677CE7B9-0003-4845-87B7-4FABD7ACD82F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -113,12 +113,6 @@
     <t>Jan 2025 - Dec 2025 (Apr 26)</t>
   </si>
   <si>
-    <t>Mar 2025 (14/10/24)</t>
-  </si>
-  <si>
-    <t>Mar 2026 (Autumn 26)</t>
-  </si>
-  <si>
     <t>&lt;a href = 'https://explore-education-statistics.service.gov.uk/find-statistics/16-18-destination-measures'&gt;16-18 destination measures&lt;/a&gt;</t>
   </si>
   <si>
@@ -168,6 +162,12 @@
   </si>
   <si>
     <t>Aug 2025 -  Jul 2026 (24/25 learners) (Oct 27)</t>
+  </si>
+  <si>
+    <t>Mar 2026 (24 September 2026)</t>
+  </si>
+  <si>
+    <t>Mar 2027 (Autumn 27)</t>
   </si>
 </sst>
 </file>
@@ -556,14 +556,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6050695-7AD5-4EAF-ACCC-796FB129457A}">
   <dimension ref="A1:H15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="86.7265625" customWidth="1"/>
-    <col min="2" max="2" width="39.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.36328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="86.7109375" customWidth="1"/>
+    <col min="2" max="2" width="39.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="41" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="41.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -577,7 +577,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>19</v>
       </c>
@@ -585,13 +585,13 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="125" customHeight="1" x14ac:dyDescent="0.35">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="125.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>18</v>
       </c>
@@ -599,13 +599,13 @@
         <v>4</v>
       </c>
       <c r="C3" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D3" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
@@ -613,56 +613,56 @@
         <v>4</v>
       </c>
       <c r="C4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D4" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="55" customHeight="1" x14ac:dyDescent="0.35">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>17</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" t="s">
         <v>31</v>
       </c>
-      <c r="C5" t="s">
-        <v>33</v>
-      </c>
       <c r="D5" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="83.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="83.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" t="s">
         <v>32</v>
       </c>
-      <c r="C6" t="s">
-        <v>33</v>
-      </c>
-      <c r="D6" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="83.5" customHeight="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="7" spans="1:8" ht="83.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D7" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="H7" s="4"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -673,10 +673,10 @@
         <v>24</v>
       </c>
       <c r="D8" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -684,13 +684,13 @@
         <v>10</v>
       </c>
       <c r="C9" t="s">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="D9" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>20</v>
       </c>
@@ -698,13 +698,13 @@
         <v>10</v>
       </c>
       <c r="C10" t="s">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="D10" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -712,41 +712,41 @@
         <v>9</v>
       </c>
       <c r="C11" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D11" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>14</v>
       </c>
       <c r="B13" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.35">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>21</v>
       </c>
@@ -754,13 +754,13 @@
         <v>22</v>
       </c>
       <c r="C14" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D14" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>15</v>
       </c>

</xml_diff>

<commit_message>
Add in NEET/not know 16-17 percentage data as a metric. Add in data informtion and caveats.
</commit_message>
<xml_diff>
--- a/Data/3-1_DataTable/DataTable.xlsx
+++ b/Data/3-1_DataTable/DataTable.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jscott8\R Projects\lsip_dashboard\Data\3-1_DataTable\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://educationgovuk-my.sharepoint.com/personal/paul_james_education_gov_uk/Documents/Documents/RProjects/lsip_dashboard/Data/3-1_DataTable/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{908255BD-55F3-4F2B-B2DD-9D3823E090BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="13_ncr:1_{908255BD-55F3-4F2B-B2DD-9D3823E090BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2F74358A-9F87-4782-9D17-75F368F158FA}"/>
   <bookViews>
-    <workbookView xWindow="1530" yWindow="10690" windowWidth="22780" windowHeight="14540" xr2:uid="{677CE7B9-0003-4845-87B7-4FABD7ACD82F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{677CE7B9-0003-4845-87B7-4FABD7ACD82F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="48">
   <si>
     <t>Data​</t>
   </si>
@@ -168,6 +168,18 @@
   </si>
   <si>
     <t>Mar 2027 (Autumn 27)</t>
+  </si>
+  <si>
+    <t>&lt;a href='https://explore-education-statistics.service.gov.uk/find-statistics/participation-in-education-training-and-neet-age-16-to-17-by-local-authority/2025-26'&gt;Participation in education, training and NEET age 16 to 17 by local authority&lt;/a&gt;</t>
+  </si>
+  <si>
+    <t>March 2026 (2/06/26)</t>
+  </si>
+  <si>
+    <t>March 2027 (July 2027)</t>
+  </si>
+  <si>
+    <t>16-17 NEET/not known by sex, SEND and ethnicity</t>
   </si>
 </sst>
 </file>
@@ -555,15 +567,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6050695-7AD5-4EAF-ACCC-796FB129457A}">
-  <dimension ref="A1:H15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:H16"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="86.7109375" customWidth="1"/>
-    <col min="2" max="2" width="39.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="86.7265625" customWidth="1"/>
+    <col min="2" max="2" width="39.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="41.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="41.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -577,7 +589,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>19</v>
       </c>
@@ -591,7 +603,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="125.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" ht="125.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>18</v>
       </c>
@@ -605,7 +617,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
@@ -619,7 +631,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" ht="55" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>17</v>
       </c>
@@ -633,7 +645,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="83.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="83.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
@@ -647,7 +659,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="83.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="83.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>39</v>
       </c>
@@ -662,7 +674,7 @@
       </c>
       <c r="H7" s="4"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -676,7 +688,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -690,7 +702,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>20</v>
       </c>
@@ -704,7 +716,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -718,7 +730,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -732,7 +744,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>14</v>
       </c>
@@ -746,7 +758,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>21</v>
       </c>
@@ -760,7 +772,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>15</v>
       </c>
@@ -772,6 +784,20 @@
       </c>
       <c r="D15" t="s">
         <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>47</v>
+      </c>
+      <c r="B16" t="s">
+        <v>44</v>
+      </c>
+      <c r="C16" t="s">
+        <v>45</v>
+      </c>
+      <c r="D16" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update job adverts data
</commit_message>
<xml_diff>
--- a/Data/3-1_DataTable/DataTable.xlsx
+++ b/Data/3-1_DataTable/DataTable.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jscott8\R Projects\lsip_dashboard\Data\3-1_DataTable\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://educationgovuk-my.sharepoint.com/personal/paul_james_education_gov_uk/Documents/Documents/RProjects/lsip_dashboard/Data/3-1_DataTable/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{908255BD-55F3-4F2B-B2DD-9D3823E090BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{908255BD-55F3-4F2B-B2DD-9D3823E090BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E9EB3021-68C8-49B0-9242-EED4D7960CE9}"/>
   <bookViews>
-    <workbookView xWindow="1530" yWindow="10690" windowWidth="22780" windowHeight="14540" xr2:uid="{677CE7B9-0003-4845-87B7-4FABD7ACD82F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{677CE7B9-0003-4845-87B7-4FABD7ACD82F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -140,12 +140,6 @@
     <t>April 2025 - Mar 2026 (TBC)</t>
   </si>
   <si>
-    <t>Jul 2026 (21/08/26)</t>
-  </si>
-  <si>
-    <t>August 2026 (Sep 2026)</t>
-  </si>
-  <si>
     <t>April 2025 - Mar 2026 (Sep 26)</t>
   </si>
   <si>
@@ -168,6 +162,12 @@
   </si>
   <si>
     <t>Mar 2027 (Autumn 27)</t>
+  </si>
+  <si>
+    <t>Sep 2026 (23/10/26)</t>
+  </si>
+  <si>
+    <t>Oct 2026 (Nov 2026)</t>
   </si>
 </sst>
 </file>
@@ -556,14 +556,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6050695-7AD5-4EAF-ACCC-796FB129457A}">
   <dimension ref="A1:H15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="86.7109375" customWidth="1"/>
-    <col min="2" max="2" width="39.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="86.7265625" customWidth="1"/>
+    <col min="2" max="2" width="39.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="41.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="41.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -577,7 +577,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>19</v>
       </c>
@@ -585,13 +585,13 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="125.1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="125.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>18</v>
       </c>
@@ -599,13 +599,13 @@
         <v>4</v>
       </c>
       <c r="C3" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D3" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
@@ -613,13 +613,13 @@
         <v>4</v>
       </c>
       <c r="C4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D4" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="55" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>17</v>
       </c>
@@ -633,7 +633,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="83.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="83.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
@@ -647,12 +647,12 @@
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="83.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="83.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C7" t="s">
         <v>31</v>
@@ -662,7 +662,7 @@
       </c>
       <c r="H7" s="4"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -676,7 +676,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -684,13 +684,13 @@
         <v>10</v>
       </c>
       <c r="C9" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D9" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>20</v>
       </c>
@@ -698,13 +698,13 @@
         <v>10</v>
       </c>
       <c r="C10" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D10" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -718,7 +718,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -726,13 +726,13 @@
         <v>26</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>14</v>
       </c>
@@ -740,13 +740,13 @@
         <v>25</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>21</v>
       </c>
@@ -754,13 +754,13 @@
         <v>22</v>
       </c>
       <c r="C14" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="D14" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>15</v>
       </c>

</xml_diff>